<commit_message>
[Feat] Embedded .bas into excel file
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Khang\Documents\Github\Debt-Calculation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9C25106-2521-4498-8383-15DE3528CF0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D80E83C-78A3-4DF9-A0C8-9596C69E0513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="19440" windowHeight="10440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -379,12 +379,6 @@
   </cellStyleXfs>
   <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
@@ -583,6 +577,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -718,314 +718,314 @@
   <dimension ref="A1:K28"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="4" width="19" style="9" customWidth="1"/>
-    <col min="5" max="5" width="19" style="79" customWidth="1"/>
-    <col min="6" max="6" width="16" style="5" customWidth="1"/>
-    <col min="7" max="7" width="13.85546875" style="5" customWidth="1"/>
-    <col min="8" max="11" width="11.5703125" style="6"/>
-    <col min="12" max="16384" width="11.5703125" style="7"/>
+    <col min="1" max="4" width="19" style="7" customWidth="1"/>
+    <col min="5" max="5" width="19" style="77" customWidth="1"/>
+    <col min="6" max="6" width="16" style="3" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" style="3" customWidth="1"/>
+    <col min="8" max="11" width="11.5703125" style="4"/>
+    <col min="12" max="16384" width="11.5703125" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="10"/>
-    </row>
-    <row r="3" spans="1:11" s="15" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="11"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="13" t="s">
+      <c r="E2" s="8"/>
+    </row>
+    <row r="3" spans="1:11" s="13" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="9"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-    </row>
-    <row r="4" spans="1:11" s="20" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="16" t="s">
+      <c r="D3" s="12"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" s="18" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="18" t="s">
+      <c r="B4" s="15"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="19"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-    </row>
-    <row r="5" spans="1:11" s="20" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="16" t="s">
+      <c r="E4" s="17"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" s="18" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="18" t="s">
+      <c r="B5" s="15"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="21"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-    </row>
-    <row r="6" spans="1:11" s="20" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="16" t="s">
+      <c r="E5" s="19"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" s="18" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
     </row>
     <row r="7" spans="1:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="17"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="18" t="s">
+      <c r="B7" s="15"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="24"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
+      <c r="E7" s="22"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
     </row>
     <row r="8" spans="1:11" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="10"/>
+      <c r="A8" s="23"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="8"/>
     </row>
     <row r="9" spans="1:11" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="4"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="28"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="29"/>
-    </row>
-    <row r="11" spans="1:11" s="35" customFormat="1" ht="27" x14ac:dyDescent="0.25">
-      <c r="A11" s="30" t="s">
+      <c r="A10" s="26"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="27"/>
+    </row>
+    <row r="11" spans="1:11" s="33" customFormat="1" ht="27" x14ac:dyDescent="0.25">
+      <c r="A11" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="31" t="s">
+      <c r="B11" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="32" t="s">
+      <c r="C11" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="31" t="s">
+      <c r="D11" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="33" t="s">
+      <c r="E11" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="F11" s="34"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="34"/>
-      <c r="I11" s="34"/>
-      <c r="J11" s="34"/>
-      <c r="K11" s="34"/>
-    </row>
-    <row r="12" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="36"/>
-      <c r="B12" s="37"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="39"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-    </row>
-    <row r="13" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="40"/>
-      <c r="B13" s="41"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="43"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-    </row>
-    <row r="14" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="40"/>
-      <c r="B14" s="41"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="43"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="32"/>
+      <c r="K11" s="32"/>
+    </row>
+    <row r="12" spans="1:11" s="18" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="34"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="37"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13" spans="1:11" s="18" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="38"/>
+      <c r="B13" s="39"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="41"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" s="18" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="38"/>
+      <c r="B14" s="39"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="41"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
     </row>
     <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="44"/>
-      <c r="B15" s="45"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
+      <c r="A15" s="42"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
     </row>
     <row r="16" spans="1:11" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="4"/>
-    </row>
-    <row r="17" spans="1:11" s="51" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="47"/>
-      <c r="B17" s="48"/>
-      <c r="C17" s="49"/>
-      <c r="D17" s="49"/>
-      <c r="E17" s="50"/>
-    </row>
-    <row r="18" spans="1:11" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="52"/>
-      <c r="B18" s="53"/>
-      <c r="C18" s="54"/>
-      <c r="D18" s="55"/>
-      <c r="E18" s="56"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:11" s="49" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="45"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="48"/>
+    </row>
+    <row r="18" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="50"/>
+      <c r="B18" s="51"/>
+      <c r="C18" s="52"/>
+      <c r="D18" s="53"/>
+      <c r="E18" s="54"/>
     </row>
     <row r="19" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="57"/>
-      <c r="B19" s="53"/>
-      <c r="C19" s="54"/>
-      <c r="D19" s="58"/>
-      <c r="E19" s="59"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="7"/>
-      <c r="J19" s="7"/>
-      <c r="K19" s="7"/>
+      <c r="A19" s="55"/>
+      <c r="B19" s="51"/>
+      <c r="C19" s="52"/>
+      <c r="D19" s="56"/>
+      <c r="E19" s="57"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
     </row>
     <row r="20" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="60"/>
-      <c r="B20" s="61" t="s">
+      <c r="A20" s="58"/>
+      <c r="B20" s="59" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="62"/>
-      <c r="D20" s="61" t="s">
+      <c r="C20" s="60"/>
+      <c r="D20" s="59" t="s">
         <v>16</v>
       </c>
-      <c r="E20" s="63"/>
+      <c r="E20" s="61"/>
     </row>
     <row r="21" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="25"/>
-      <c r="B21" s="64" t="s">
+      <c r="A21" s="23"/>
+      <c r="B21" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="12"/>
-      <c r="D21" s="64" t="s">
+      <c r="C21" s="10"/>
+      <c r="D21" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="E21" s="10"/>
+      <c r="E21" s="8"/>
     </row>
     <row r="22" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="25"/>
-      <c r="E22" s="10"/>
+      <c r="A22" s="23"/>
+      <c r="E22" s="8"/>
     </row>
     <row r="23" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="25"/>
-      <c r="E23" s="10"/>
+      <c r="A23" s="23"/>
+      <c r="E23" s="8"/>
     </row>
     <row r="24" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="25"/>
-      <c r="E24" s="10"/>
+      <c r="A24" s="23"/>
+      <c r="E24" s="8"/>
     </row>
     <row r="25" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="25"/>
-      <c r="E25" s="10"/>
-    </row>
-    <row r="26" spans="1:11" s="68" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="65"/>
-      <c r="B26" s="66"/>
-      <c r="C26" s="66"/>
-      <c r="D26" s="66"/>
-      <c r="E26" s="67"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
-    </row>
-    <row r="27" spans="1:11" s="68" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="69"/>
-      <c r="B27" s="70"/>
-      <c r="C27" s="71" t="s">
+      <c r="A25" s="23"/>
+      <c r="E25" s="8"/>
+    </row>
+    <row r="26" spans="1:11" s="66" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="63"/>
+      <c r="B26" s="64"/>
+      <c r="C26" s="64"/>
+      <c r="D26" s="64"/>
+      <c r="E26" s="65"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+    </row>
+    <row r="27" spans="1:11" s="66" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="67"/>
+      <c r="B27" s="68"/>
+      <c r="C27" s="69" t="s">
         <v>18</v>
       </c>
-      <c r="D27" s="72"/>
-      <c r="E27" s="73"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
+      <c r="D27" s="70"/>
+      <c r="E27" s="71"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
     </row>
     <row r="28" spans="1:11" ht="16.149999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="74"/>
-      <c r="B28" s="75"/>
-      <c r="C28" s="76" t="s">
+      <c r="A28" s="72"/>
+      <c r="B28" s="73"/>
+      <c r="C28" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="D28" s="77"/>
-      <c r="E28" s="78"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
+      <c r="D28" s="75"/>
+      <c r="E28" s="76"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>